<commit_message>
Add points for 2bi32jvwjtru3nrkulzx3ip04_playerlog
</commit_message>
<xml_diff>
--- a/bnc-streamlit-app/data/points/2bi32jvwjtru3nrkulzx3ip04_playerlog.xlsx
+++ b/bnc-streamlit-app/data/points/2bi32jvwjtru3nrkulzx3ip04_playerlog.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BG24"/>
+  <dimension ref="A1:BG33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -766,10 +766,12 @@
           <t>795i2d5jpiflpdzfh6pb9l8t1</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="n">
+        <v>2</v>
+      </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K2" t="inlineStr"/>
@@ -780,14 +782,14 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="n">
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
@@ -795,7 +797,7 @@
         </is>
       </c>
       <c r="S2" t="n">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
@@ -825,7 +827,7 @@
         <v>0</v>
       </c>
       <c r="AG2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH2" t="inlineStr"/>
       <c r="AI2" t="inlineStr"/>
@@ -835,7 +837,7 @@
         <v>0</v>
       </c>
       <c r="AM2" t="n">
-        <v>21</v>
+        <v>90</v>
       </c>
       <c r="AN2" t="n">
         <v>0</v>
@@ -850,7 +852,7 @@
         <v>0</v>
       </c>
       <c r="AR2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS2" t="n">
         <v>1</v>
@@ -951,14 +953,14 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="n">
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
@@ -966,7 +968,7 @@
         </is>
       </c>
       <c r="S3" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
@@ -990,10 +992,10 @@
         <v>0</v>
       </c>
       <c r="AE3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AF3" t="n">
-        <v>-0.2</v>
+        <v>-1</v>
       </c>
       <c r="AG3" t="n">
         <v>1</v>
@@ -1004,21 +1006,21 @@
         </is>
       </c>
       <c r="AI3" t="n">
-        <v>-0.15206872</v>
+        <v>-0.58149482</v>
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>-0.22</t>
+          <t>-1.15</t>
         </is>
       </c>
       <c r="AK3" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="AL3" t="n">
         <v>0</v>
       </c>
       <c r="AM3" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="AN3" t="n">
         <v>0</v>
@@ -1027,7 +1029,7 @@
         <v>0</v>
       </c>
       <c r="AP3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ3" t="n">
         <v>0</v>
@@ -1036,13 +1038,13 @@
         <v>0</v>
       </c>
       <c r="AS3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AT3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AU3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AV3" t="n">
         <v>0</v>
@@ -1073,7 +1075,7 @@
         <v>0</v>
       </c>
       <c r="BF3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG3" t="n">
         <v>0</v>
@@ -1134,14 +1136,14 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="n">
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
@@ -1149,7 +1151,7 @@
         </is>
       </c>
       <c r="S4" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
@@ -1173,10 +1175,10 @@
         <v>0</v>
       </c>
       <c r="AE4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AF4" t="n">
-        <v>-0.2</v>
+        <v>-1</v>
       </c>
       <c r="AG4" t="n">
         <v>1</v>
@@ -1187,21 +1189,21 @@
         </is>
       </c>
       <c r="AI4" t="n">
-        <v>-0.20532038</v>
+        <v>-0.5918857900000001</v>
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
-          <t>-0.27</t>
+          <t>-1.16</t>
         </is>
       </c>
       <c r="AK4" t="n">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="AL4" t="n">
         <v>0</v>
       </c>
       <c r="AM4" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="AN4" t="n">
         <v>0</v>
@@ -1216,16 +1218,16 @@
         <v>0</v>
       </c>
       <c r="AR4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AS4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AT4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AV4" t="n">
         <v>0</v>
@@ -1234,7 +1236,7 @@
         <v>0</v>
       </c>
       <c r="AX4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY4" t="n">
         <v>0</v>
@@ -1317,14 +1319,14 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="n">
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
@@ -1332,7 +1334,7 @@
         </is>
       </c>
       <c r="S5" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
@@ -1356,10 +1358,10 @@
         <v>0</v>
       </c>
       <c r="AE5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AF5" t="n">
-        <v>-0.05</v>
+        <v>-0.25</v>
       </c>
       <c r="AG5" t="n">
         <v>1</v>
@@ -1370,21 +1372,21 @@
         </is>
       </c>
       <c r="AI5" t="n">
-        <v>-0.05248771</v>
+        <v>-0.48002968</v>
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>-0.12</t>
+          <t>-1.05</t>
         </is>
       </c>
       <c r="AK5" t="n">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="AL5" t="n">
         <v>0</v>
       </c>
       <c r="AM5" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="AN5" t="n">
         <v>0</v>
@@ -1393,31 +1395,31 @@
         <v>0</v>
       </c>
       <c r="AP5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ5" t="n">
         <v>0</v>
       </c>
       <c r="AR5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AS5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AT5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW5" t="n">
         <v>0</v>
       </c>
       <c r="AX5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY5" t="n">
         <v>0</v>
@@ -1439,7 +1441,7 @@
         <v>0</v>
       </c>
       <c r="BF5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG5" t="n">
         <v>0</v>
@@ -1553,15 +1555,15 @@
         </is>
       </c>
       <c r="AI6" t="n">
-        <v>-0.5386280000000001</v>
+        <v>-0.53077489</v>
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
-          <t>-0.60</t>
+          <t>-1.10</t>
         </is>
       </c>
       <c r="AK6" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="AL6" t="n">
         <v>0</v>
@@ -1683,14 +1685,14 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="n">
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
@@ -1698,7 +1700,7 @@
         </is>
       </c>
       <c r="S7" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
@@ -1722,10 +1724,10 @@
         <v>0</v>
       </c>
       <c r="AE7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AF7" t="n">
-        <v>-0.2</v>
+        <v>-1</v>
       </c>
       <c r="AG7" t="n">
         <v>1</v>
@@ -1736,21 +1738,21 @@
         </is>
       </c>
       <c r="AI7" t="n">
-        <v>-0.34342934</v>
+        <v>-0.3473503900000001</v>
       </c>
       <c r="AJ7" t="inlineStr">
         <is>
-          <t>-0.41</t>
+          <t>-0.91</t>
         </is>
       </c>
       <c r="AK7" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="AL7" t="n">
         <v>0</v>
       </c>
       <c r="AM7" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="AN7" t="n">
         <v>0</v>
@@ -1765,19 +1767,19 @@
         <v>1</v>
       </c>
       <c r="AR7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AS7" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="AT7" t="n">
         <v>0</v>
       </c>
       <c r="AU7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW7" t="n">
         <v>0</v>
@@ -1921,15 +1923,15 @@
         </is>
       </c>
       <c r="AI8" t="n">
-        <v>-0.03222285000000001</v>
+        <v>-0.04513626</v>
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
-          <t>-0.10</t>
+          <t>-0.61</t>
         </is>
       </c>
       <c r="AK8" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="AL8" t="n">
         <v>0</v>
@@ -2037,10 +2039,12 @@
           <t>dmnk8dz6w8n4fcso88fuvusfe</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
+      <c r="I9" t="n">
+        <v>2</v>
+      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K9" t="inlineStr"/>
@@ -2051,14 +2055,14 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>21</v>
+        <v>66</v>
       </c>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="n">
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>21</v>
+        <v>66</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
@@ -2066,7 +2070,7 @@
         </is>
       </c>
       <c r="S9" t="n">
-        <v>21</v>
+        <v>66</v>
       </c>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
@@ -2090,13 +2094,13 @@
         <v>0</v>
       </c>
       <c r="AE9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AF9" t="n">
-        <v>-0.05</v>
+        <v>-0.15</v>
       </c>
       <c r="AG9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
@@ -2104,21 +2108,21 @@
         </is>
       </c>
       <c r="AI9" t="n">
-        <v>0.001113809999999993</v>
+        <v>-0.4542304</v>
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>-0.07</t>
+          <t>-1.02</t>
         </is>
       </c>
       <c r="AK9" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="AL9" t="n">
         <v>0</v>
       </c>
       <c r="AM9" t="n">
-        <v>21</v>
+        <v>66</v>
       </c>
       <c r="AN9" t="n">
         <v>0</v>
@@ -2130,10 +2134,10 @@
         <v>0</v>
       </c>
       <c r="AQ9" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AR9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AS9" t="n">
         <v>0</v>
@@ -2142,7 +2146,7 @@
         <v>0</v>
       </c>
       <c r="AU9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV9" t="n">
         <v>0</v>
@@ -2173,7 +2177,7 @@
         <v>0</v>
       </c>
       <c r="BF9" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="BG9" t="n">
         <v>0</v>
@@ -2220,10 +2224,12 @@
           <t>3a96rdsu1qqtsmiaae10vbyi2</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
+      <c r="I10" t="n">
+        <v>2</v>
+      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K10" t="inlineStr"/>
@@ -2234,14 +2240,14 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>21</v>
+        <v>57</v>
       </c>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="n">
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>21</v>
+        <v>57</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
@@ -2249,7 +2255,7 @@
         </is>
       </c>
       <c r="S10" t="n">
-        <v>21</v>
+        <v>57</v>
       </c>
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
@@ -2273,13 +2279,13 @@
         <v>0</v>
       </c>
       <c r="AE10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AF10" t="n">
         <v>0</v>
       </c>
       <c r="AG10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH10" t="inlineStr">
         <is>
@@ -2287,21 +2293,21 @@
         </is>
       </c>
       <c r="AI10" t="n">
-        <v>-0.01869629</v>
+        <v>0.20085118</v>
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
-          <t>-0.08</t>
+          <t>-0.36</t>
         </is>
       </c>
       <c r="AK10" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="AL10" t="n">
         <v>0</v>
       </c>
       <c r="AM10" t="n">
-        <v>21</v>
+        <v>57</v>
       </c>
       <c r="AN10" t="n">
         <v>0</v>
@@ -2310,22 +2316,22 @@
         <v>0</v>
       </c>
       <c r="AP10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ10" t="n">
         <v>0</v>
       </c>
       <c r="AR10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV10" t="n">
         <v>0</v>
@@ -2356,7 +2362,7 @@
         <v>0</v>
       </c>
       <c r="BF10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG10" t="n">
         <v>0</v>
@@ -2403,10 +2409,12 @@
           <t>m9kg2l0d9lr6r3k0hu8hqgb8</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" t="n">
+        <v>2</v>
+      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K11" t="inlineStr"/>
@@ -2417,14 +2425,14 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>21</v>
+        <v>57</v>
       </c>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="n">
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>21</v>
+        <v>57</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
@@ -2432,7 +2440,7 @@
         </is>
       </c>
       <c r="S11" t="n">
-        <v>21</v>
+        <v>57</v>
       </c>
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
@@ -2456,13 +2464,13 @@
         <v>0</v>
       </c>
       <c r="AE11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AF11" t="n">
-        <v>-0.05</v>
+        <v>-0.1</v>
       </c>
       <c r="AG11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
@@ -2470,21 +2478,21 @@
         </is>
       </c>
       <c r="AI11" t="n">
-        <v>0.06182128</v>
+        <v>0.09903228000000003</v>
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>-0.00</t>
+          <t>-0.47</t>
         </is>
       </c>
       <c r="AK11" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="AL11" t="n">
         <v>0</v>
       </c>
       <c r="AM11" t="n">
-        <v>21</v>
+        <v>57</v>
       </c>
       <c r="AN11" t="n">
         <v>0</v>
@@ -2499,7 +2507,7 @@
         <v>0</v>
       </c>
       <c r="AR11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AS11" t="n">
         <v>0</v>
@@ -2514,7 +2522,7 @@
         <v>0</v>
       </c>
       <c r="AW11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX11" t="n">
         <v>0</v>
@@ -2539,7 +2547,7 @@
         <v>0</v>
       </c>
       <c r="BF11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG11" t="n">
         <v>0</v>
@@ -2600,7 +2608,7 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -2611,7 +2619,7 @@
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
@@ -2627,7 +2635,7 @@
         </is>
       </c>
       <c r="U12" t="n">
-        <v>5.3</v>
+        <v>80.3</v>
       </c>
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr"/>
@@ -2649,7 +2657,7 @@
         <v>0</v>
       </c>
       <c r="AE12" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AF12" t="n">
         <v>0</v>
@@ -2663,21 +2671,21 @@
         </is>
       </c>
       <c r="AI12" t="n">
-        <v>0.0006288900000000017</v>
+        <v>0.36591357</v>
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
-          <t>-0.07</t>
+          <t>-0.20</t>
         </is>
       </c>
       <c r="AK12" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="AL12" t="n">
         <v>0</v>
       </c>
       <c r="AM12" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="AN12" t="n">
         <v>0</v>
@@ -2689,19 +2697,19 @@
         <v>0</v>
       </c>
       <c r="AQ12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AR12" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AS12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AT12" t="n">
         <v>0</v>
       </c>
       <c r="AU12" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AV12" t="n">
         <v>0</v>
@@ -2732,7 +2740,7 @@
         <v>0</v>
       </c>
       <c r="BF12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BG12" t="n">
         <v>0</v>
@@ -2797,14 +2805,14 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>6</v>
+        <v>81</v>
       </c>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="n">
         <v>15</v>
       </c>
       <c r="Q13" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
@@ -2812,7 +2820,7 @@
         </is>
       </c>
       <c r="S13" t="n">
-        <v>6</v>
+        <v>81</v>
       </c>
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
@@ -2836,10 +2844,10 @@
         <v>0</v>
       </c>
       <c r="AE13" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AF13" t="n">
-        <v>-0</v>
+        <v>-0.8</v>
       </c>
       <c r="AG13" t="n">
         <v>1</v>
@@ -2850,21 +2858,21 @@
         </is>
       </c>
       <c r="AI13" t="n">
-        <v>0.25745448</v>
+        <v>0.06053385999999983</v>
       </c>
       <c r="AJ13" t="inlineStr">
         <is>
-          <t>+0.19</t>
+          <t>-0.51</t>
         </is>
       </c>
       <c r="AK13" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="AL13" t="n">
         <v>15</v>
       </c>
       <c r="AM13" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="AN13" t="n">
         <v>0</v>
@@ -2879,19 +2887,19 @@
         <v>0</v>
       </c>
       <c r="AR13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS13" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AT13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AW13" t="n">
         <v>0</v>
@@ -2933,37 +2941,37 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2wk1549tkz80oet8226euj7jp</t>
+          <t>7u6a9femhquay3jnk6ysgiwx9</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>M. Diaw</t>
+          <t>Ali Yousif</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>23</t>
+          <t xml:space="preserve"> 13</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>GK</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>c6u4h9wy88ymj6whiz93jknv9</t>
+          <t>eyr7cp5tb5wtexg3ljluvus4p</t>
         </is>
       </c>
       <c r="I14" t="inlineStr"/>
@@ -2972,30 +2980,34 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
+      <c r="K14" t="n">
+        <v>57</v>
+      </c>
+      <c r="L14" t="n">
+        <v>2</v>
+      </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="N14" t="n">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="n">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="Q14" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>GK</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="S14" t="n">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
@@ -3007,35 +3019,47 @@
       <c r="AA14" t="inlineStr"/>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>2wk1549tkz80oet8226euj7jp</t>
+          <t>7u6a9femhquay3jnk6ysgiwx9</t>
         </is>
       </c>
       <c r="AC14" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Iraq</t>
         </is>
       </c>
       <c r="AD14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE14" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AF14" t="n">
         <v>0</v>
       </c>
       <c r="AG14" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH14" t="inlineStr"/>
-      <c r="AI14" t="inlineStr"/>
-      <c r="AJ14" t="inlineStr"/>
-      <c r="AK14" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="AH14" t="inlineStr">
+        <is>
+          <t>Ali Yousif</t>
+        </is>
+      </c>
+      <c r="AI14" t="n">
+        <v>0.20207851</v>
+      </c>
+      <c r="AJ14" t="inlineStr">
+        <is>
+          <t>-0.36</t>
+        </is>
+      </c>
+      <c r="AK14" t="n">
+        <v>17</v>
+      </c>
       <c r="AL14" t="n">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="AM14" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="AN14" t="n">
         <v>0</v>
@@ -3047,19 +3071,19 @@
         <v>0</v>
       </c>
       <c r="AQ14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AT14" t="n">
         <v>0</v>
       </c>
       <c r="AU14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV14" t="n">
         <v>0</v>
@@ -3090,7 +3114,7 @@
         <v>0</v>
       </c>
       <c r="BF14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG14" t="n">
         <v>0</v>
@@ -3104,12 +3128,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2wk1549tkz80oet8226euj7jp</t>
+          <t>7u6a9femhquay3jnk6ysgiwx9</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>K. Diatta</t>
+          <t>Ahmed Maknzi</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -3119,22 +3143,22 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>f5j3vhj805xtkos7l538u0d7t</t>
+          <t>ckvrq3cddvlk3rgxr5i0ykz55</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
@@ -3143,30 +3167,34 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
+      <c r="K15" t="n">
+        <v>57</v>
+      </c>
+      <c r="L15" t="n">
+        <v>2</v>
+      </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="N15" t="n">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="n">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="Q15" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="S15" t="n">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr"/>
@@ -3178,47 +3206,47 @@
       <c r="AA15" t="inlineStr"/>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>2wk1549tkz80oet8226euj7jp</t>
+          <t>7u6a9femhquay3jnk6ysgiwx9</t>
         </is>
       </c>
       <c r="AC15" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Iraq</t>
         </is>
       </c>
       <c r="AD15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AF15" t="n">
-        <v>-0</v>
+        <v>-0.15</v>
       </c>
       <c r="AG15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH15" t="inlineStr">
         <is>
-          <t>K. Diatta</t>
+          <t>Ahmed Maknzi</t>
         </is>
       </c>
       <c r="AI15" t="n">
-        <v>0.03662801</v>
+        <v>0.04880411999999997</v>
       </c>
       <c r="AJ15" t="inlineStr">
         <is>
-          <t>-0.03</t>
+          <t>-0.52</t>
         </is>
       </c>
       <c r="AK15" t="n">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="AL15" t="n">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="AM15" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="AN15" t="n">
         <v>0</v>
@@ -3230,19 +3258,19 @@
         <v>0</v>
       </c>
       <c r="AQ15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AR15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AS15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AT15" t="n">
         <v>0</v>
       </c>
       <c r="AU15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AV15" t="n">
         <v>0</v>
@@ -3273,7 +3301,7 @@
         <v>0</v>
       </c>
       <c r="BF15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="BG15" t="n">
         <v>0</v>
@@ -3287,37 +3315,37 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2wk1549tkz80oet8226euj7jp</t>
+          <t>7u6a9femhquay3jnk6ysgiwx9</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>I. Jakobs</t>
+          <t>K. Yakob</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 14</t>
+          <t xml:space="preserve"> 19</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>RCM(2)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>9bqv99e39z86mn7dq3wnyt90p</t>
+          <t>asfu3i70ss0wqmdenqpx37p7u</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
@@ -3326,30 +3354,34 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
+      <c r="K16" t="n">
+        <v>66</v>
+      </c>
+      <c r="L16" t="n">
+        <v>2</v>
+      </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="N16" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="Q16" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>RCM(2)</t>
         </is>
       </c>
       <c r="S16" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
@@ -3361,47 +3393,47 @@
       <c r="AA16" t="inlineStr"/>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>2wk1549tkz80oet8226euj7jp</t>
+          <t>7u6a9femhquay3jnk6ysgiwx9</t>
         </is>
       </c>
       <c r="AC16" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Iraq</t>
         </is>
       </c>
       <c r="AD16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AF16" t="n">
-        <v>-0</v>
+        <v>-0.1</v>
       </c>
       <c r="AG16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH16" t="inlineStr">
         <is>
-          <t>I. Jakobs</t>
+          <t>K. Yakob</t>
         </is>
       </c>
       <c r="AI16" t="n">
-        <v>-0.08590808</v>
+        <v>0.08920843999999997</v>
       </c>
       <c r="AJ16" t="inlineStr">
         <is>
-          <t>-0.15</t>
+          <t>-0.48</t>
         </is>
       </c>
       <c r="AK16" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="AL16" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="AM16" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="AN16" t="n">
         <v>0</v>
@@ -3413,19 +3445,19 @@
         <v>0</v>
       </c>
       <c r="AQ16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AR16" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AS16" t="n">
         <v>0</v>
       </c>
       <c r="AT16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV16" t="n">
         <v>0</v>
@@ -3456,7 +3488,7 @@
         <v>0</v>
       </c>
       <c r="BF16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BG16" t="n">
         <v>0</v>
@@ -3470,37 +3502,37 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2wk1549tkz80oet8226euj7jp</t>
+          <t>7u6a9femhquay3jnk6ysgiwx9</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>I. Gueye</t>
+          <t>Jalal Hassan</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 5</t>
+          <t xml:space="preserve"> 12</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>CM(3)</t>
+          <t>GK</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>ceerfv28fygp7m2euv5n5uu39</t>
+          <t>co041fmv8xhrrtoyp2fuxzsnp</t>
         </is>
       </c>
       <c r="I17" t="inlineStr"/>
@@ -3509,30 +3541,34 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
+      <c r="K17" t="n">
+        <v>45</v>
+      </c>
+      <c r="L17" t="n">
+        <v>2</v>
+      </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="N17" t="n">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="Q17" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>CM(3)</t>
+          <t>GK</t>
         </is>
       </c>
       <c r="S17" t="n">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
@@ -3544,47 +3580,35 @@
       <c r="AA17" t="inlineStr"/>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>2wk1549tkz80oet8226euj7jp</t>
+          <t>7u6a9femhquay3jnk6ysgiwx9</t>
         </is>
       </c>
       <c r="AC17" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Iraq</t>
         </is>
       </c>
       <c r="AD17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE17" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AF17" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AG17" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH17" t="inlineStr">
-        <is>
-          <t>I. Gueye</t>
-        </is>
-      </c>
-      <c r="AI17" t="n">
-        <v>-0.003990429999999996</v>
-      </c>
-      <c r="AJ17" t="inlineStr">
-        <is>
-          <t>-0.07</t>
-        </is>
-      </c>
-      <c r="AK17" t="n">
-        <v>13</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="AH17" t="inlineStr"/>
+      <c r="AI17" t="inlineStr"/>
+      <c r="AJ17" t="inlineStr"/>
+      <c r="AK17" t="inlineStr"/>
       <c r="AL17" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="AM17" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="AN17" t="n">
         <v>0</v>
@@ -3599,7 +3623,7 @@
         <v>0</v>
       </c>
       <c r="AR17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS17" t="n">
         <v>0</v>
@@ -3608,10 +3632,10 @@
         <v>0</v>
       </c>
       <c r="AU17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AW17" t="n">
         <v>0</v>
@@ -3658,17 +3682,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>A. Seck</t>
+          <t>M. Diaw</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 4</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>RCB(2)</t>
+          <t>GK</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -3678,12 +3702,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>4gglrx5t4kgdqqc51tgfjgz4l</t>
+          <t>c6u4h9wy88ymj6whiz93jknv9</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
@@ -3700,22 +3724,22 @@
         </is>
       </c>
       <c r="N18" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="n">
         <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>RCB(2)</t>
+          <t>GK</t>
         </is>
       </c>
       <c r="S18" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr"/>
@@ -3736,53 +3760,41 @@
         </is>
       </c>
       <c r="AD18" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AE18" t="n">
         <v>0</v>
       </c>
       <c r="AF18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AG18" t="n">
         <v>1</v>
       </c>
-      <c r="AH18" t="inlineStr">
-        <is>
-          <t>A. Seck</t>
-        </is>
-      </c>
-      <c r="AI18" t="n">
-        <v>0.71229136</v>
-      </c>
-      <c r="AJ18" t="inlineStr">
-        <is>
-          <t>+0.65</t>
-        </is>
-      </c>
-      <c r="AK18" t="n">
-        <v>2</v>
-      </c>
+      <c r="AH18" t="inlineStr"/>
+      <c r="AI18" t="inlineStr"/>
+      <c r="AJ18" t="inlineStr"/>
+      <c r="AK18" t="inlineStr"/>
       <c r="AL18" t="n">
         <v>0</v>
       </c>
       <c r="AM18" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="AN18" t="n">
         <v>0</v>
       </c>
       <c r="AO18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ18" t="n">
         <v>0</v>
       </c>
       <c r="AR18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AS18" t="n">
         <v>0</v>
@@ -3800,7 +3812,7 @@
         <v>0</v>
       </c>
       <c r="AX18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AY18" t="n">
         <v>0</v>
@@ -3822,7 +3834,7 @@
         <v>0</v>
       </c>
       <c r="BF18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BG18" t="n">
         <v>0</v>
@@ -3841,17 +3853,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>M. Niakhaté</t>
+          <t>K. Diatta</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 19</t>
+          <t xml:space="preserve"> 15</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>LCB(2)</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -3861,12 +3873,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>9rf5uk6c2wce30b9wkmu3iuad</t>
+          <t>f5j3vhj805xtkos7l538u0d7t</t>
         </is>
       </c>
       <c r="I19" t="inlineStr"/>
@@ -3883,22 +3895,22 @@
         </is>
       </c>
       <c r="N19" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="n">
         <v>0</v>
       </c>
       <c r="Q19" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>LCB(2)</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="S19" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="T19" t="inlineStr"/>
       <c r="U19" t="inlineStr"/>
@@ -3919,38 +3931,38 @@
         </is>
       </c>
       <c r="AD19" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AE19" t="n">
         <v>0</v>
       </c>
       <c r="AF19" t="n">
-        <v>-0</v>
+        <v>0.4</v>
       </c>
       <c r="AG19" t="n">
         <v>1</v>
       </c>
       <c r="AH19" t="inlineStr">
         <is>
-          <t>M. Niakhaté</t>
+          <t>K. Diatta</t>
         </is>
       </c>
       <c r="AI19" t="n">
-        <v>0.02824415</v>
+        <v>1.56523619</v>
       </c>
       <c r="AJ19" t="inlineStr">
         <is>
-          <t>-0.04</t>
+          <t>+1.00</t>
         </is>
       </c>
       <c r="AK19" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="AL19" t="n">
         <v>0</v>
       </c>
       <c r="AM19" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="AN19" t="n">
         <v>0</v>
@@ -3959,13 +3971,13 @@
         <v>0</v>
       </c>
       <c r="AP19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AR19" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AS19" t="n">
         <v>0</v>
@@ -3974,7 +3986,7 @@
         <v>0</v>
       </c>
       <c r="AU19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AV19" t="n">
         <v>0</v>
@@ -4005,7 +4017,7 @@
         <v>0</v>
       </c>
       <c r="BF19" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="BG19" t="n">
         <v>0</v>
@@ -4024,17 +4036,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>H. Diarra</t>
+          <t>I. Jakobs</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 21</t>
+          <t xml:space="preserve"> 14</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>RCM(3)</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -4044,12 +4056,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>egtyl4noukbjkm1va1i11e87o</t>
+          <t>9bqv99e39z86mn7dq3wnyt90p</t>
         </is>
       </c>
       <c r="I20" t="inlineStr"/>
@@ -4066,22 +4078,22 @@
         </is>
       </c>
       <c r="N20" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="n">
         <v>0</v>
       </c>
       <c r="Q20" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>RCM(3)</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="S20" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
@@ -4102,56 +4114,56 @@
         </is>
       </c>
       <c r="AD20" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AE20" t="n">
         <v>0</v>
       </c>
       <c r="AF20" t="n">
-        <v>-0</v>
+        <v>0.4</v>
       </c>
       <c r="AG20" t="n">
         <v>1</v>
       </c>
       <c r="AH20" t="inlineStr">
         <is>
-          <t>H. Diarra</t>
+          <t>I. Jakobs</t>
         </is>
       </c>
       <c r="AI20" t="n">
-        <v>0.9677131999999999</v>
+        <v>0.74847317</v>
       </c>
       <c r="AJ20" t="inlineStr">
         <is>
-          <t>+0.90</t>
+          <t>+0.18</t>
         </is>
       </c>
       <c r="AK20" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="AL20" t="n">
         <v>0</v>
       </c>
       <c r="AM20" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="AN20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO20" t="n">
         <v>0</v>
       </c>
       <c r="AP20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR20" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AS20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT20" t="n">
         <v>0</v>
@@ -4163,7 +4175,7 @@
         <v>0</v>
       </c>
       <c r="AW20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AX20" t="n">
         <v>0</v>
@@ -4188,7 +4200,7 @@
         <v>0</v>
       </c>
       <c r="BF20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BG20" t="n">
         <v>0</v>
@@ -4207,17 +4219,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>L. Camara</t>
+          <t>I. Gueye</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 8</t>
+          <t xml:space="preserve"> 5</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>LCM(3)</t>
+          <t>CM(3)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -4227,12 +4239,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>8eq4c5cotvem9ae9uzb2yezo4</t>
+          <t>ceerfv28fygp7m2euv5n5uu39</t>
         </is>
       </c>
       <c r="I21" t="inlineStr"/>
@@ -4249,25 +4261,35 @@
         </is>
       </c>
       <c r="N21" t="n">
-        <v>21</v>
-      </c>
-      <c r="O21" t="inlineStr"/>
+        <v>96</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>RCM(2)</t>
+        </is>
+      </c>
       <c r="P21" t="n">
         <v>0</v>
       </c>
       <c r="Q21" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>LCM(3)</t>
+          <t>CM(3)</t>
         </is>
       </c>
       <c r="S21" t="n">
-        <v>21</v>
-      </c>
-      <c r="T21" t="inlineStr"/>
-      <c r="U21" t="inlineStr"/>
+        <v>57.9</v>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>RCM(2)</t>
+        </is>
+      </c>
+      <c r="U21" t="n">
+        <v>38.1</v>
+      </c>
       <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr"/>
       <c r="X21" t="inlineStr"/>
@@ -4285,65 +4307,65 @@
         </is>
       </c>
       <c r="AD21" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AE21" t="n">
         <v>0</v>
       </c>
       <c r="AF21" t="n">
-        <v>-0</v>
+        <v>0.1</v>
       </c>
       <c r="AG21" t="n">
         <v>1</v>
       </c>
       <c r="AH21" t="inlineStr">
         <is>
-          <t>L. Camara</t>
+          <t>I. Gueye</t>
         </is>
       </c>
       <c r="AI21" t="n">
-        <v>0.31171672</v>
+        <v>0.98878365</v>
       </c>
       <c r="AJ21" t="inlineStr">
         <is>
-          <t>+0.25</t>
+          <t>+0.42</t>
         </is>
       </c>
       <c r="AK21" t="n">
+        <v>8</v>
+      </c>
+      <c r="AL21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM21" t="n">
+        <v>96</v>
+      </c>
+      <c r="AN21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP21" t="n">
         <v>4</v>
       </c>
-      <c r="AL21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM21" t="n">
-        <v>21</v>
-      </c>
-      <c r="AN21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP21" t="n">
-        <v>2</v>
-      </c>
       <c r="AQ21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AR21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AS21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT21" t="n">
         <v>0</v>
       </c>
       <c r="AU21" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AV21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW21" t="n">
         <v>0</v>
@@ -4371,7 +4393,7 @@
         <v>0</v>
       </c>
       <c r="BF21" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="BG21" t="n">
         <v>0</v>
@@ -4390,17 +4412,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>I. Sarr</t>
+          <t>A. Seck</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 18</t>
+          <t xml:space="preserve"> 4</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>RCB(2)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -4410,18 +4432,20 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>44s112hd02w1i2ucvai9jy7e1</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr"/>
+          <t>4gglrx5t4kgdqqc51tgfjgz4l</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>2</v>
+      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K22" t="inlineStr"/>
@@ -4432,22 +4456,22 @@
         </is>
       </c>
       <c r="N22" t="n">
-        <v>21</v>
+        <v>57</v>
       </c>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="n">
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>21</v>
+        <v>57</v>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>RCB(2)</t>
         </is>
       </c>
       <c r="S22" t="n">
-        <v>21</v>
+        <v>57</v>
       </c>
       <c r="T22" t="inlineStr"/>
       <c r="U22" t="inlineStr"/>
@@ -4468,57 +4492,57 @@
         </is>
       </c>
       <c r="AD22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE22" t="n">
         <v>0</v>
       </c>
       <c r="AF22" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AG22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH22" t="inlineStr">
         <is>
-          <t>I. Sarr</t>
+          <t>A. Seck</t>
         </is>
       </c>
       <c r="AI22" t="n">
-        <v>0.56249234</v>
+        <v>0.8605490199999999</v>
       </c>
       <c r="AJ22" t="inlineStr">
         <is>
-          <t>+0.50</t>
+          <t>+0.29</t>
         </is>
       </c>
       <c r="AK22" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM22" t="n">
+        <v>57</v>
+      </c>
+      <c r="AN22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR22" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS22" t="n">
         <v>3</v>
       </c>
-      <c r="AL22" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM22" t="n">
-        <v>21</v>
-      </c>
-      <c r="AN22" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO22" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP22" t="n">
-        <v>1</v>
-      </c>
-      <c r="AQ22" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR22" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS22" t="n">
-        <v>1</v>
-      </c>
       <c r="AT22" t="n">
         <v>0</v>
       </c>
@@ -4532,7 +4556,7 @@
         <v>0</v>
       </c>
       <c r="AX22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY22" t="n">
         <v>0</v>
@@ -4573,17 +4597,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>I. Mbaye</t>
+          <t>M. Niakhaté</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 20</t>
+          <t xml:space="preserve"> 19</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>LCB(2)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -4593,12 +4617,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>20eqyvyrgtafzssdh0zaehdsk</t>
+          <t>9rf5uk6c2wce30b9wkmu3iuad</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
@@ -4615,22 +4639,22 @@
         </is>
       </c>
       <c r="N23" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="n">
         <v>0</v>
       </c>
       <c r="Q23" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>LCB(2)</t>
         </is>
       </c>
       <c r="S23" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
@@ -4651,38 +4675,38 @@
         </is>
       </c>
       <c r="AD23" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AE23" t="n">
         <v>0</v>
       </c>
       <c r="AF23" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="AG23" t="n">
         <v>1</v>
       </c>
       <c r="AH23" t="inlineStr">
         <is>
-          <t>I. Mbaye</t>
+          <t>M. Niakhaté</t>
         </is>
       </c>
       <c r="AI23" t="n">
-        <v>0.03971764</v>
+        <v>0.91148507</v>
       </c>
       <c r="AJ23" t="inlineStr">
         <is>
-          <t>-0.03</t>
+          <t>+0.35</t>
         </is>
       </c>
       <c r="AK23" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AL23" t="n">
         <v>0</v>
       </c>
       <c r="AM23" t="n">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="AN23" t="n">
         <v>0</v>
@@ -4694,16 +4718,16 @@
         <v>0</v>
       </c>
       <c r="AQ23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR23" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AS23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU23" t="n">
         <v>0</v>
@@ -4737,7 +4761,7 @@
         <v>0</v>
       </c>
       <c r="BF23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG23" t="n">
         <v>0</v>
@@ -4756,17 +4780,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>S. Mané</t>
+          <t>H. Diarra</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 10</t>
+          <t xml:space="preserve"> 21</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>LW</t>
+          <t>RCM(3)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -4776,18 +4800,20 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>cotiiu6mjkfx5xa63nhfbdf4l</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr"/>
+          <t>egtyl4noukbjkm1va1i11e87o</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>2</v>
+      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K24" t="inlineStr"/>
@@ -4798,22 +4824,22 @@
         </is>
       </c>
       <c r="N24" t="n">
-        <v>21</v>
+        <v>56</v>
       </c>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="n">
         <v>0</v>
       </c>
       <c r="Q24" t="n">
-        <v>21</v>
+        <v>56</v>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>LW</t>
+          <t>RCM(3)</t>
         </is>
       </c>
       <c r="S24" t="n">
-        <v>21</v>
+        <v>56</v>
       </c>
       <c r="T24" t="inlineStr"/>
       <c r="U24" t="inlineStr"/>
@@ -4834,100 +4860,1783 @@
         </is>
       </c>
       <c r="AD24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE24" t="n">
         <v>0</v>
       </c>
       <c r="AF24" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AG24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH24" t="inlineStr">
         <is>
+          <t>H. Diarra</t>
+        </is>
+      </c>
+      <c r="AI24" t="n">
+        <v>1.38680018</v>
+      </c>
+      <c r="AJ24" t="inlineStr">
+        <is>
+          <t>+0.82</t>
+        </is>
+      </c>
+      <c r="AK24" t="n">
+        <v>7</v>
+      </c>
+      <c r="AL24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM24" t="n">
+        <v>56</v>
+      </c>
+      <c r="AN24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD24" t="inlineStr"/>
+      <c r="BE24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF24" t="n">
+        <v>3</v>
+      </c>
+      <c r="BG24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2bi32jvwjtru3nrkulzx3ip04</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>L. Camara</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 8</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LCM(3)</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>8eq4c5cotvem9ae9uzb2yezo4</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>2</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N25" t="n">
+        <v>56</v>
+      </c>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>56</v>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>LCM(3)</t>
+        </is>
+      </c>
+      <c r="S25" t="n">
+        <v>56</v>
+      </c>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr"/>
+      <c r="W25" t="inlineStr"/>
+      <c r="X25" t="inlineStr"/>
+      <c r="Y25" t="inlineStr"/>
+      <c r="Z25" t="inlineStr"/>
+      <c r="AA25" t="inlineStr"/>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="AD25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF25" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AG25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH25" t="inlineStr">
+        <is>
+          <t>L. Camara</t>
+        </is>
+      </c>
+      <c r="AI25" t="n">
+        <v>1.42627109</v>
+      </c>
+      <c r="AJ25" t="inlineStr">
+        <is>
+          <t>+0.86</t>
+        </is>
+      </c>
+      <c r="AK25" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM25" t="n">
+        <v>56</v>
+      </c>
+      <c r="AN25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP25" t="n">
+        <v>4</v>
+      </c>
+      <c r="AQ25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR25" t="n">
+        <v>7</v>
+      </c>
+      <c r="AS25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD25" t="inlineStr"/>
+      <c r="BE25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF25" t="n">
+        <v>5</v>
+      </c>
+      <c r="BG25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2bi32jvwjtru3nrkulzx3ip04</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>I. Sarr</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 18</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>44s112hd02w1i2ucvai9jy7e1</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>2</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N26" t="n">
+        <v>80</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>80</v>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="S26" t="n">
+        <v>57.9</v>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="U26" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="V26" t="inlineStr"/>
+      <c r="W26" t="inlineStr"/>
+      <c r="X26" t="inlineStr"/>
+      <c r="Y26" t="inlineStr"/>
+      <c r="Z26" t="inlineStr"/>
+      <c r="AA26" t="inlineStr"/>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="AD26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG26" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH26" t="inlineStr">
+        <is>
+          <t>I. Sarr</t>
+        </is>
+      </c>
+      <c r="AI26" t="n">
+        <v>2.6042367</v>
+      </c>
+      <c r="AJ26" t="inlineStr">
+        <is>
+          <t>+2.04</t>
+        </is>
+      </c>
+      <c r="AK26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM26" t="n">
+        <v>80</v>
+      </c>
+      <c r="AN26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP26" t="n">
+        <v>2</v>
+      </c>
+      <c r="AQ26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AS26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV26" t="n">
+        <v>2</v>
+      </c>
+      <c r="AW26" t="n">
+        <v>2</v>
+      </c>
+      <c r="AX26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD26" t="inlineStr"/>
+      <c r="BE26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF26" t="n">
+        <v>4</v>
+      </c>
+      <c r="BG26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2bi32jvwjtru3nrkulzx3ip04</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>I. Mbaye</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 20</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>20eqyvyrgtafzssdh0zaehdsk</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>2</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N27" t="n">
+        <v>56</v>
+      </c>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>56</v>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="S27" t="n">
+        <v>56</v>
+      </c>
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr"/>
+      <c r="W27" t="inlineStr"/>
+      <c r="X27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr"/>
+      <c r="AA27" t="inlineStr"/>
+      <c r="AB27" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="AD27" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG27" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH27" t="inlineStr">
+        <is>
+          <t>I. Mbaye</t>
+        </is>
+      </c>
+      <c r="AI27" t="n">
+        <v>0.4446521</v>
+      </c>
+      <c r="AJ27" t="inlineStr">
+        <is>
+          <t>-0.12</t>
+        </is>
+      </c>
+      <c r="AK27" t="n">
+        <v>13</v>
+      </c>
+      <c r="AL27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM27" t="n">
+        <v>56</v>
+      </c>
+      <c r="AN27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ27" t="n">
+        <v>3</v>
+      </c>
+      <c r="AR27" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD27" t="inlineStr"/>
+      <c r="BE27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF27" t="n">
+        <v>4</v>
+      </c>
+      <c r="BG27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2bi32jvwjtru3nrkulzx3ip04</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
           <t>S. Mané</t>
         </is>
       </c>
-      <c r="AI24" t="n">
-        <v>0.14041115</v>
-      </c>
-      <c r="AJ24" t="inlineStr">
-        <is>
-          <t>+0.07</t>
-        </is>
-      </c>
-      <c r="AK24" t="n">
+      <c r="D28" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 10</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LW</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>cotiiu6mjkfx5xa63nhfbdf4l</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N28" t="n">
+        <v>96</v>
+      </c>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>96</v>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>LW</t>
+        </is>
+      </c>
+      <c r="S28" t="n">
+        <v>96</v>
+      </c>
+      <c r="T28" t="inlineStr"/>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr"/>
+      <c r="W28" t="inlineStr"/>
+      <c r="X28" t="inlineStr"/>
+      <c r="Y28" t="inlineStr"/>
+      <c r="Z28" t="inlineStr"/>
+      <c r="AA28" t="inlineStr"/>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="AD28" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH28" t="inlineStr">
+        <is>
+          <t>S. Mané</t>
+        </is>
+      </c>
+      <c r="AI28" t="n">
+        <v>1.49544624</v>
+      </c>
+      <c r="AJ28" t="inlineStr">
+        <is>
+          <t>+0.93</t>
+        </is>
+      </c>
+      <c r="AK28" t="n">
+        <v>5</v>
+      </c>
+      <c r="AL28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM28" t="n">
+        <v>96</v>
+      </c>
+      <c r="AN28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP28" t="n">
+        <v>4</v>
+      </c>
+      <c r="AQ28" t="n">
+        <v>3</v>
+      </c>
+      <c r="AR28" t="n">
+        <v>4</v>
+      </c>
+      <c r="AS28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD28" t="inlineStr">
+        <is>
+          <t>FWD</t>
+        </is>
+      </c>
+      <c r="BE28" t="n">
+        <v>4</v>
+      </c>
+      <c r="BF28" t="n">
+        <v>8</v>
+      </c>
+      <c r="BG28" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2bi32jvwjtru3nrkulzx3ip04</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>P. Ciss</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>RCB(2)</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>1ho7koiegfhsuevuum2meibu2</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K29" t="n">
+        <v>57</v>
+      </c>
+      <c r="L29" t="n">
+        <v>2</v>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N29" t="n">
+        <v>39</v>
+      </c>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="n">
+        <v>57</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>96</v>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>RCB(2)</t>
+        </is>
+      </c>
+      <c r="S29" t="n">
+        <v>39</v>
+      </c>
+      <c r="T29" t="inlineStr"/>
+      <c r="U29" t="inlineStr"/>
+      <c r="V29" t="inlineStr"/>
+      <c r="W29" t="inlineStr"/>
+      <c r="X29" t="inlineStr"/>
+      <c r="Y29" t="inlineStr"/>
+      <c r="Z29" t="inlineStr"/>
+      <c r="AA29" t="inlineStr"/>
+      <c r="AB29" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="AD29" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF29" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AG29" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH29" t="inlineStr">
+        <is>
+          <t>P. Ciss</t>
+        </is>
+      </c>
+      <c r="AI29" t="n">
+        <v>0.38358335</v>
+      </c>
+      <c r="AJ29" t="inlineStr">
+        <is>
+          <t>-0.18</t>
+        </is>
+      </c>
+      <c r="AK29" t="n">
+        <v>14</v>
+      </c>
+      <c r="AL29" t="n">
+        <v>57</v>
+      </c>
+      <c r="AM29" t="n">
+        <v>96</v>
+      </c>
+      <c r="AN29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD29" t="inlineStr"/>
+      <c r="BE29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF29" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG29" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2bi32jvwjtru3nrkulzx3ip04</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>A. Diao</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 7</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>13uxs8820y7mi31fsw1i0qxw4</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K30" t="n">
+        <v>80</v>
+      </c>
+      <c r="L30" t="n">
+        <v>2</v>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N30" t="n">
+        <v>16</v>
+      </c>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>96</v>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="S30" t="n">
+        <v>16</v>
+      </c>
+      <c r="T30" t="inlineStr"/>
+      <c r="U30" t="inlineStr"/>
+      <c r="V30" t="inlineStr"/>
+      <c r="W30" t="inlineStr"/>
+      <c r="X30" t="inlineStr"/>
+      <c r="Y30" t="inlineStr"/>
+      <c r="Z30" t="inlineStr"/>
+      <c r="AA30" t="inlineStr"/>
+      <c r="AB30" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="AC30" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="AD30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG30" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH30" t="inlineStr">
+        <is>
+          <t>A. Diao</t>
+        </is>
+      </c>
+      <c r="AI30" t="n">
+        <v>0.27037775</v>
+      </c>
+      <c r="AJ30" t="inlineStr">
+        <is>
+          <t>-0.30</t>
+        </is>
+      </c>
+      <c r="AK30" t="n">
+        <v>16</v>
+      </c>
+      <c r="AL30" t="n">
+        <v>80</v>
+      </c>
+      <c r="AM30" t="n">
+        <v>96</v>
+      </c>
+      <c r="AN30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ30" t="n">
+        <v>3</v>
+      </c>
+      <c r="AR30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD30" t="inlineStr"/>
+      <c r="BE30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF30" t="n">
+        <v>3</v>
+      </c>
+      <c r="BG30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2bi32jvwjtru3nrkulzx3ip04</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>N. Jackson</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 11</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>amcwh6w0brmkttg4uc5qm6z9w</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K31" t="n">
+        <v>56</v>
+      </c>
+      <c r="L31" t="n">
+        <v>2</v>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N31" t="n">
+        <v>40</v>
+      </c>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="n">
+        <v>56</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>96</v>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="S31" t="n">
+        <v>40</v>
+      </c>
+      <c r="T31" t="inlineStr"/>
+      <c r="U31" t="inlineStr"/>
+      <c r="V31" t="inlineStr"/>
+      <c r="W31" t="inlineStr"/>
+      <c r="X31" t="inlineStr"/>
+      <c r="Y31" t="inlineStr"/>
+      <c r="Z31" t="inlineStr"/>
+      <c r="AA31" t="inlineStr"/>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="AD31" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG31" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH31" t="inlineStr">
+        <is>
+          <t>N. Jackson</t>
+        </is>
+      </c>
+      <c r="AI31" t="n">
+        <v>0.8215644</v>
+      </c>
+      <c r="AJ31" t="inlineStr">
+        <is>
+          <t>+0.26</t>
+        </is>
+      </c>
+      <c r="AK31" t="n">
+        <v>11</v>
+      </c>
+      <c r="AL31" t="n">
+        <v>56</v>
+      </c>
+      <c r="AM31" t="n">
+        <v>96</v>
+      </c>
+      <c r="AN31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW31" t="n">
+        <v>2</v>
+      </c>
+      <c r="AX31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD31" t="inlineStr"/>
+      <c r="BE31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF31" t="n">
+        <v>3</v>
+      </c>
+      <c r="BG31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2bi32jvwjtru3nrkulzx3ip04</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>I. Ndiaye</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 13</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>3dm2bfuoyips4rbj0vhvbp9be</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K32" t="n">
+        <v>56</v>
+      </c>
+      <c r="L32" t="n">
+        <v>2</v>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N32" t="n">
+        <v>40</v>
+      </c>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="n">
+        <v>56</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>96</v>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="S32" t="n">
+        <v>40</v>
+      </c>
+      <c r="T32" t="inlineStr"/>
+      <c r="U32" t="inlineStr"/>
+      <c r="V32" t="inlineStr"/>
+      <c r="W32" t="inlineStr"/>
+      <c r="X32" t="inlineStr"/>
+      <c r="Y32" t="inlineStr"/>
+      <c r="Z32" t="inlineStr"/>
+      <c r="AA32" t="inlineStr"/>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="AD32" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG32" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH32" t="inlineStr">
+        <is>
+          <t>I. Ndiaye</t>
+        </is>
+      </c>
+      <c r="AI32" t="n">
+        <v>2.73545584</v>
+      </c>
+      <c r="AJ32" t="inlineStr">
+        <is>
+          <t>+2.17</t>
+        </is>
+      </c>
+      <c r="AK32" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL32" t="n">
+        <v>56</v>
+      </c>
+      <c r="AM32" t="n">
+        <v>96</v>
+      </c>
+      <c r="AN32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP32" t="n">
+        <v>2</v>
+      </c>
+      <c r="AQ32" t="n">
+        <v>5</v>
+      </c>
+      <c r="AR32" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW32" t="n">
+        <v>2</v>
+      </c>
+      <c r="AX32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD32" t="inlineStr"/>
+      <c r="BE32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF32" t="n">
+        <v>9</v>
+      </c>
+      <c r="BG32" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2bi32jvwjtru3nrkulzx3ip04</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>P. Gueye</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 26</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LCM(2)</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>ekm47qd8w1x0456lm1tmf5re1</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K33" t="n">
+        <v>56</v>
+      </c>
+      <c r="L33" t="n">
+        <v>2</v>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N33" t="n">
+        <v>40</v>
+      </c>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="n">
+        <v>56</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>96</v>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>LCM(2)</t>
+        </is>
+      </c>
+      <c r="S33" t="n">
+        <v>40</v>
+      </c>
+      <c r="T33" t="inlineStr"/>
+      <c r="U33" t="inlineStr"/>
+      <c r="V33" t="inlineStr"/>
+      <c r="W33" t="inlineStr"/>
+      <c r="X33" t="inlineStr"/>
+      <c r="Y33" t="inlineStr"/>
+      <c r="Z33" t="inlineStr"/>
+      <c r="AA33" t="inlineStr"/>
+      <c r="AB33" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="AD33" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AG33" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH33" t="inlineStr">
+        <is>
+          <t>P. Gueye</t>
+        </is>
+      </c>
+      <c r="AI33" t="n">
+        <v>3.65019534</v>
+      </c>
+      <c r="AJ33" t="inlineStr">
+        <is>
+          <t>+3.08</t>
+        </is>
+      </c>
+      <c r="AK33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL33" t="n">
+        <v>56</v>
+      </c>
+      <c r="AM33" t="n">
+        <v>96</v>
+      </c>
+      <c r="AN33" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP33" t="n">
+        <v>3</v>
+      </c>
+      <c r="AQ33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR33" t="n">
+        <v>4</v>
+      </c>
+      <c r="AS33" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW33" t="n">
+        <v>3</v>
+      </c>
+      <c r="AX33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD33" t="inlineStr"/>
+      <c r="BE33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF33" t="n">
         <v>6</v>
       </c>
-      <c r="AL24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM24" t="n">
-        <v>21</v>
-      </c>
-      <c r="AN24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW24" t="n">
-        <v>1</v>
-      </c>
-      <c r="AX24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD24" t="inlineStr">
-        <is>
-          <t>FWD</t>
-        </is>
-      </c>
-      <c r="BE24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF24" t="n">
-        <v>1</v>
-      </c>
-      <c r="BG24" t="n">
-        <v>1</v>
+      <c r="BG33" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>